<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.003-07 Le lapin et la soupe
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-07.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-07.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut faire visiter le parc puis le jardin à son lapin, avant la soupe. À chaque départ, il reprend ce qu'il faut pour que le lapin rentre.</t>
+          <t>Un toc sec vient du métal. Sur le bord, un éclat de casserole brille. Amir veut que le lapin voie le parc, maintenant, avant la soupe. Il pousse manteau et doudou dans le seau : trop lourd, ça bascule. Il refuse de forcer, reprend seau, manteau, lapin. Merci vécu. Au jardin, l'odeur de soupe appelle. Il refuse de foncer. Dans l'eau de la gourde, l'éclat pointe le lapin. Ils rentrent. L'éclat de casserole et le fil de vapeur se regardent.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Dans la cuisine, la casserole sent la carotte. Elle est encore tiède. La cuillère en bois repose sur le torchon. La soupe attend pour ce soir, Amir. Ça sent bon. Oui. Carotte et poireau. Maman pose le couvercle. Ça fait un petit toc. On va au parc, maintenant. Oui. Le lapin vient. Il voyage. Ils ferment la porte. La soupe reste à la maison. En ce moment, Amir est au parc. Le vent fraîchit. Maman s'assoit sur le banc. Amir a un seau rouge. Il a un manteau vert. Il a son doudou lapin. Le manteau est sur le banc. Le seau, c'est sa valise. Je te vois. Amir verse le sable. Ça fait chh. Le vent soulève un peu de poussière. Le lapin attend dans l'herbe. L'herbe chatouille. Le vent fraîchit. On rentre. Le lapin n'a pas tout vu. Il verra le jardin, après. On reprend ses affaires, avant de partir. Amir s'arrête. Il cherche le seau près du bac. Il le prend. J'ai la valise. Bien. Il cherche le manteau sur le banc. Il le prend. Le manteau vert. Et le lapin ? Il cherche le doudou dans l'herbe. L'herbe chatouille. Il le prend. Le lapin aussi. Merci, Amir. Maintenant Amir a tout. Ils rentrent un moment. Plus tard, ils jouent au jardin. L'odeur de soupe est encore là. Elle passe sous la porte. Amir a une gourde. Il a une casquette. Il a encore le doudou. Je bois. Doucement. L'eau est fraîche. Une feuille tourne près du pied. Le jardin, il a vu. On rentre. La soupe est prête. Le lapin aussi. Avant de partir, on reprend ses affaires. La gourde a roulé près de la feuille. La casquette est sur une chaise. Le lapin est dans l'herbe courte.</t>
+          <t>Un toc sec vient du métal. Le couvercle de la casserole repose de travers. Le torchon sent le poireau, et la carotte. La cuillère en bois laisse une trace humide. La soupe attend pour ce soir, Amir. Ça sent bon. Tu sens la carotte ? Oui, maman. Et le poireau. Maman pose le couvercle. Ça fait un petit toc. Un fil de vapeur glisse sur le bord. Sur le bord, un éclat de casserole brille. Il brille, maman. C'est un éclat de casserole, Amir. Le doudou lapin attend sur la chaise. Le lapin veut le parc, maintenant ! La soupe reste ici. On y va ? Oui, avec sa valise. Ils ferment la porte de la cuisine. La soupe reste à la maison. En ce moment, Amir est au parc. Le vent fraîchit sur le bac des valises. Maman s'assoit sur le banc. Amir a un seau rouge. Son manteau vert attend sur le banc. Le lapin attend dans l'herbe. Le seau, c'est sa valise. Je te vois. Amir verse le sable. Ça fait chh. Il voyage, maman. Le vent fraîchit. On rentre. Le lapin n'a pas tout vu ! Le jardin, maintenant ! Après, oui. Amir veut tout mettre d'un coup. Il pousse le manteau dans le seau. Il pousse le lapin par-dessus. Le seau bascule, trop lourd. Le sable coule sur ses chaussures. Ça reste coincé ! Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu reprends le seau ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Dans la cuisine, la casserole sent la carotte. Elle est encore tiède. La cuillère en bois repose sur le torchon. La soupe attend pour ce soir, Amir. Ça sent bon. Oui. Carotte et poireau. Maman pose le couvercle. Ça fait un petit toc. On va au parc, maintenant. Oui. Le lapin vient. Il voyage. Ils ferment la porte. La soupe reste à la maison. En ce moment, Amir est au parc. Le vent fraîchit. Maman s'assoit sur le banc. Amir a un seau rouge. Il a un manteau vert. Il a son doudou lapin. Le manteau est sur le banc. Le seau, c'est sa valise. Je te vois. Amir verse le sable. Ça fait chh. Le vent soulève un peu de poussière. Le lapin attend dans l'herbe. L'herbe chatouille. Le vent fraîchit. On rentre. Le lapin n'a pas tout vu. Il verra le jardin, après. On reprend ses affaires, avant de partir. Amir s'arrête. Il cherche le seau près du bac. Il le prend. J'ai la valise. Bien. Il cherche le manteau sur le banc. Il le prend. Le manteau vert. Et le lapin ? Il cherche le doudou dans l'herbe. L'herbe chatouille. Il le prend. Le lapin aussi. Merci, Amir. Maintenant Amir a tout. Ils rentrent un moment. Plus tard, ils jouent au jardin. L'odeur de soupe est encore là. Elle passe sous la porte. Amir a une gourde. Il a une casquette. Il a encore le doudou. Je bois. Doucement. L'eau est fraîche. Une feuille tourne près du pied. Le jardin, il a vu. On rentre. La soupe est prête. Le lapin aussi. Avant de partir, on reprend ses affaires. La gourde a roulé près de la feuille. La casquette est sur une chaise. Le lapin est dans l'herbe courte.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un toc sec vient du métal. Le couvercle de la casserole repose de travers. Le torchon sent le poireau, et la carotte. La cuillère en bois laisse une trace humide. La soupe attend pour ce soir, Amir. Ça sent bon. Tu sens la carotte ? Oui, maman. Et le poireau. Maman pose le couvercle. Ça fait un petit toc. Un fil de vapeur glisse sur le bord. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de casserole&lt;/emphasis&gt; brille. Il brille, maman. C'est un éclat de casserole, Amir. Le doudou lapin attend sur la chaise. Le lapin veut le parc, maintenant ! La soupe reste ici. On y va ? Oui, avec sa valise. Ils ferment la porte de la cuisine. La soupe reste à la maison. En ce moment, Amir est au parc. Le vent fraîchit sur le bac des valises. Maman s'assoit sur le banc. Amir a un seau rouge. Son manteau vert attend sur le banc. Le lapin attend dans l'herbe. Le seau, c'est sa valise. Je te vois. Amir verse le sable. Ça fait chh. Il voyage, maman. Le vent fraîchit. On rentre. Le lapin n'a pas tout vu ! Le jardin, maintenant ! Après, oui. Amir veut tout mettre d'un coup. Il pousse le manteau dans le seau. Il pousse le lapin par-dessus. Le seau bascule, trop lourd. Le sable coule sur ses chaussures. Ça reste coincé ! Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu reprends le seau ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Benoît a joué longtemps au parc. Maman est sur le banc. Benoît a un seau rouge. Il a un manteau vert. Il a son doudou lapin. Le vent fraîchit. Maman dit : on rentre. Maman dit : on va &lt;emphasis&gt;reprendre&lt;/emphasis&gt; ses affaires, avant de partir. Benoît s'arrête. Il cherche le seau près du bac. Il le prend. Il cherche le manteau sur le banc. Il le prend. Il cherche le doudou dans l'herbe. L'herbe chatouille. Il le prend. Maintenant Benoît a tout. Maman dit : merci. Plus tard, ils jouent au jardin. Benoît a une gourde. Il a une casquette. Il a encore le doudou. Maman dit : on rentre. Benoît se souvient. Avant de partir, on reprend ses affaires. Il cherche la gourde. Il la prend. Il cherche la casquette. Il la prend. Il cherche le doudou. Il le prend. Maman dit : tu as repris le geste. Même leçon, autre lieu. Benoît a tout. Ils marchent vers la maison. [pause]</t>
+          <t>Un toc sec vient du métal. Le couvercle de la casserole repose de travers. Le torchon sent le poireau, et la carotte. La cuillère en bois laisse une trace humide. La soupe attend pour ce soir, Amir. Ça sent bon. Tu sens la carotte ? Oui, maman. Et le poireau. Maman pose le couvercle. Ça fait un petit toc. Un fil de vapeur glisse sur le bord. Sur le bord, un &lt;emphasis&gt;éclat de casserole&lt;/emphasis&gt; brille. Il brille, maman. C'est un éclat de casserole, Amir. Le doudou lapin attend sur la chaise. Le lapin veut le parc, maintenant ! La soupe reste ici. On y va ? Oui, avec sa valise. Ils ferment la porte de la cuisine. La soupe reste à la maison. En ce moment, Amir est au parc. Le vent fraîchit sur le bac des valises. Maman s'assoit sur le banc. Amir a un seau rouge. Son manteau vert attend sur le banc. Le lapin attend dans l'herbe. Le seau, c'est sa valise. Je te vois. Amir verse le sable. Ça fait chh. Il voyage, maman. Le vent fraîchit. On rentre. Le lapin n'a pas tout vu ! Le jardin, maintenant ! Après, oui. Amir veut tout mettre d'un coup. Il pousse le manteau dans le seau. Il pousse le lapin par-dessus. Le seau bascule, trop lourd. Le sable coule sur ses chaussures. Ça reste coincé ! Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu reprends le seau ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>éclat de casserole</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,82 +1326,65 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_parc_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Dans la cuisine, la casserole sent la carotte.
-narrateur|Elle est encore tiède.
-narrateur|La cuillère en bois repose sur le torchon.
+          <t>narrateur|Un toc sec vient du métal.
+narrateur|Le couvercle de la casserole repose de travers.
+narrateur|Le torchon sent le poireau, et la carotte.
+narrateur|La cuillère en bois laisse une trace humide.
 maman|La soupe attend pour ce soir, Amir.
 enfant-m|Ça sent bon.
-maman|Oui.
-maman|Carotte et poireau.
+maman|Tu sens la carotte ?
+enfant-m|Oui, maman.
+enfant-m|Et le poireau.
 narrateur|Maman pose le couvercle.
 narrateur|Ça fait un petit toc.
-maman|On va au parc, maintenant.
-enfant-m|Oui.
-enfant-m|Le lapin vient.
-maman|Il voyage.
-narrateur|Ils ferment la porte.
+narrateur|Un fil de vapeur glisse sur le bord.
+narrateur|Sur le bord, un éclat de casserole brille.
+enfant-m|Il brille, maman.
+maman|C'est un éclat de casserole, Amir.
+narrateur|Le doudou lapin attend sur la chaise.
+enfant-m|Le lapin veut le parc, maintenant !
+maman|La soupe reste ici.
+enfant-m|On y va ?
+maman|Oui, avec sa valise.
+narrateur|Ils ferment la porte de la cuisine.
 narrateur|La soupe reste à la maison.
 narrateur|En ce moment, Amir est au parc.
-narrateur|Le vent fraîchit.
+narrateur|Le vent fraîchit sur le bac des valises.
 narrateur|Maman s'assoit sur le banc.
 narrateur|Amir a un seau rouge.
-narrateur|Il a un manteau vert.
-narrateur|Il a son doudou lapin.
-narrateur|Le manteau est sur le banc.
+narrateur|Son manteau vert attend sur le banc.
+narrateur|Le lapin attend dans l'herbe.
 enfant-m|Le seau, c'est sa valise.
 maman|Je te vois.
 narrateur|Amir verse le sable.
 narrateur|Ça fait chh.
-narrateur|Le vent soulève un peu de poussière.
-narrateur|Le lapin attend dans l'herbe.
-narrateur|L'herbe chatouille.
+enfant-m|Il voyage, maman.
 maman|Le vent fraîchit.
 maman|On rentre.
-enfant-m|Le lapin n'a pas tout vu.
-maman|Il verra le jardin, après.
-maman|On reprend ses affaires, avant de partir.
-narrateur|Amir s'arrête.
-narrateur|Il cherche le seau près du bac.
-narrateur|Il le prend.
-enfant-m|J'ai la valise.
-maman|Bien.
-narrateur|Il cherche le manteau sur le banc.
-narrateur|Il le prend.
-enfant-m|Le manteau vert.
-maman|Et le lapin ?
-narrateur|Il cherche le doudou dans l'herbe.
-narrateur|L'herbe chatouille.
-narrateur|Il le prend.
-enfant-m|Le lapin aussi.
-maman|Merci, Amir.
-narrateur|Maintenant Amir a tout.
-narrateur|Ils rentrent un moment.
-narrateur|Plus tard, ils jouent au jardin.
-narrateur|L'odeur de soupe est encore là.
-narrateur|Elle passe sous la porte.
-narrateur|Amir a une gourde.
-narrateur|Il a une casquette.
-narrateur|Il a encore le doudou.
-enfant-m|Je bois.
-maman|Doucement.
-narrateur|L'eau est fraîche.
-narrateur|Une feuille tourne près du pied.
-enfant-m|Le jardin, il a vu.
-maman|On rentre.
-maman|La soupe est prête.
-enfant-m|Le lapin aussi.
-maman|Avant de partir, on reprend ses affaires.
-narrateur|La gourde a roulé près de la feuille.
-narrateur|La casquette est sur une chaise.
-narrateur|Le lapin est dans l'herbe courte.</t>
+enfant-m|Le lapin n'a pas tout vu !
+enfant-m|Le jardin, maintenant !
+maman|Après, oui.
+narrateur|Amir veut tout mettre d'un coup.
+narrateur|Il pousse le manteau dans le seau.
+narrateur|Il pousse le lapin par-dessus.
+narrateur|Le seau bascule, trop lourd.
+narrateur|Le sable coule sur ses chaussures.
+enfant-m|Ça reste coincé !
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+maman|Tu reprends le seau ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>casserole,vapeur</t>
         </is>
       </c>
     </row>
@@ -1428,17 +1411,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Amir ?</t>
+          <t>Amir reprend le seau. Avant de partir, que fait Amir ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Amir ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir &lt;emphasis level="moderate"&gt;reprend&lt;/emphasis&gt; le seau. Avant de partir, que fait Amir ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;emphasis&gt;avant&lt;/emphasis&gt; de partir, que fait Benoît ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir &lt;emphasis&gt;reprend&lt;/emphasis&gt; le seau. Avant de partir, que fait Amir ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1501,18 +1484,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1527,38 +1510,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>reprend</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1567,28 +1550,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_reprend_avant_de_partir; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir, que fait Amir ?</t>
+          <t>narrateur|Amir reprend le seau.
+narrateur|Avant de partir, que fait Amir ?</t>
         </is>
       </c>
     </row>
@@ -1615,17 +1599,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir se souvient. Il cherche la gourde. Il la prend près de la feuille. Il cherche la casquette. Il la prend. Il cherche le doudou. Il le prend. J'ai tout. Tu as repris tes affaires. Avant de partir. Au parc, puis au jardin. Les deux fois. Bravo, Amir. Amir a tout. Ils marchent vers la maison. Le doudou est dans son bras. Tu tiens le lapin ? Oui. Il a voyagé.</t>
+          <t>Maman s'accroupit à la même hauteur. Amir refuse de tirer plus fort. Je sors le lapin. Il tire le tissu coincé, sans forcer. Le lapin glisse, un peu froid. Il était dans le seau. Tu le poses où ? Près du banc. Amir pose le lapin sur le bois. Le banc est froid sous la laine. Et le manteau ? Je le prends. Il reprend le manteau vert, sur le banc. Le tissu vert gratte un peu, aux poignets. J'ai les bras dedans. Tu as fini tes manches ? Oui, maman. Amir reprend le seau près du bac. J'ai la valise. Merci, Amir. Maman ouvre le portillon du parc. L'air frais pique les joues. On va au jardin ? Oui, le lapin va le voir.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir se souvient. Il cherche la gourde. Il la prend près de la feuille. Il cherche la casquette. Il la prend. Il cherche le doudou. Il le prend. J'ai tout. Tu as repris tes affaires. Avant de partir. Au parc, puis au jardin. Les deux fois. Bravo, Amir. Amir a tout. Ils marchent vers la maison. Le doudou est dans son bras. Tu tiens le lapin ? Oui. Il a voyagé.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman s'accroupit à la même hauteur. Amir refuse de tirer plus fort. Je sors le lapin. Il tire le tissu coincé, sans forcer. Le lapin glisse, un peu froid. Il était dans le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;. Tu le poses où ? Près du banc. Amir pose le lapin sur le bois. Le banc est froid sous la laine. Et le manteau ? Je le prends. Il reprend le manteau vert, sur le banc. Le tissu vert gratte un peu, aux poignets. J'ai les bras dedans. Tu as fini tes manches ? Oui, maman. Amir reprend le seau près du bac. J'ai la valise. Merci, Amir. Maman ouvre le portillon du parc. L'air frais pique les joues. On va au jardin ? Oui, le lapin va le voir.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Benoît a cherché. Il a repris ses affaires. C'était &lt;emphasis&gt;avant&lt;/emphasis&gt; de partir. Au parc, puis au jardin. [pause]</t>
+          <t>Maman s'accroupit à la même hauteur. Amir refuse de tirer plus fort. Je sors le lapin. Il tire le tissu coincé, sans forcer. Le lapin glisse, un peu froid. Il était dans le &lt;emphasis&gt;seau&lt;/emphasis&gt;. Tu le poses où ? Près du banc. Amir pose le lapin sur le bois. Le banc est froid sous la laine. Et le manteau ? Je le prends. Il reprend le manteau vert, sur le banc. Le tissu vert gratte un peu, aux poignets. J'ai les bras dedans. Tu as fini tes manches ? Oui, maman. Amir reprend le seau près du bac. J'ai la valise. Merci, Amir. Maman ouvre le portillon du parc. L'air frais pique les joues. On va au jardin ? Oui, le lapin va le voir. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1672,7 +1656,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1680,10 +1664,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1706,7 +1690,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>seau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1720,16 +1704,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1738,10 +1722,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1754,35 +1738,40 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=une_chose_puis_l_autre; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir se souvient.
-narrateur|Il cherche la gourde.
-narrateur|Il la prend près de la feuille.
-narrateur|Il cherche la casquette.
-narrateur|Il la prend.
-narrateur|Il cherche le doudou.
-narrateur|Il le prend.
-enfant-m|J'ai tout.
-maman|Tu as repris tes affaires.
-enfant-m|Avant de partir.
-enfant-m|Au parc, puis au jardin.
-maman|Les deux fois.
-maman|Bravo, Amir.
-narrateur|Amir a tout.
-narrateur|Ils marchent vers la maison.
-narrateur|Le doudou est dans son bras.
-maman|Tu tiens le lapin ?
-enfant-m|Oui.
-enfant-m|Il a voyagé.</t>
+          <t>narrateur|Maman s'accroupit à la même hauteur.
+narrateur|Amir refuse de tirer plus fort.
+enfant-m|Je sors le lapin.
+narrateur|Il tire le tissu coincé, sans forcer.
+narrateur|Le lapin glisse, un peu froid.
+enfant-m|Il était dans le seau.
+maman|Tu le poses où ?
+enfant-m|Près du banc.
+narrateur|Amir pose le lapin sur le bois.
+narrateur|Le banc est froid sous la laine.
+maman|Et le manteau ?
+enfant-m|Je le prends.
+narrateur|Il reprend le manteau vert, sur le banc.
+narrateur|Le tissu vert gratte un peu, aux poignets.
+enfant-m|J'ai les bras dedans.
+maman|Tu as fini tes manches ?
+enfant-m|Oui, maman.
+narrateur|Amir reprend le seau près du bac.
+enfant-m|J'ai la valise.
+maman|Merci, Amir.
+narrateur|Maman ouvre le portillon du parc.
+narrateur|L'air frais pique les joues.
+enfant-m|On va au jardin ?
+maman|Oui, le lapin va le voir.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>sable,banc</t>
         </is>
       </c>
     </row>
@@ -1809,17 +1798,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Amir marche près de maman. Le doudou est dans son bras. Ils ouvrent la porte. La soupe sent encore plus fort. Tu poses la gourde près de l'évier ? Amir pose la gourde. Il pose la casquette. Merci. Ce soir, on mange la soupe. Carotte et poireau. Oui. Amir pose le lapin sur une chaise. Il a vu le parc. Il a vu le jardin. Et maintenant, la soupe. Un peu de vapeur monte. Il goûte l'odeur. Tout doux.</t>
+          <t>Plus tard, ils jouent au jardin. L'odeur de soupe passe sous la porte. Amir a une gourde. Il a une casquette. Le lapin est dans l'herbe courte. Je bois. Doucement. L'eau est fraîche. Une feuille tourne près du pied. Le jardin, il a vu. La soupe, maintenant ! On rentre. Je cours ! Amir veut foncer vers la porte. La gourde a roulé près de la feuille. La casquette est sur une chaise basse. Le sourire d'Amir se serre. Ça serre, dans son ventre. Je n'aime pas ça. Amir refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Amir observe la gourde, écoute le jardin. Dans l'eau, un éclat blanc tremble. Comme l'éclat de casserole, maman ! Tu le vois, celui-là ? Oui, maman. Il pointe le lapin. Il contourne la feuille, lentement. Il reprend la gourde près de la feuille. Il reprend la casquette, sur la chaise. Et le lapin. Le doudou est dans son bras. Tu tiens le lapin ? Oui, il a voyagé.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Amir marche près de maman. Le doudou est dans son bras. Ils ouvrent la porte. La soupe sent encore plus fort. Tu poses la gourde près de l'évier ? Amir pose la gourde. Il pose la casquette. Merci. Ce soir, on mange la soupe. Carotte et poireau. Oui. Amir pose le lapin sur une chaise. Il a vu le parc. Il a vu le jardin. Et maintenant, la soupe. Un peu de vapeur monte. Il goûte l'odeur. Tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus tard, ils jouent au jardin. L'odeur de soupe passe sous la porte. Amir a une gourde. Il a une casquette. Le lapin est dans l'herbe courte. Je bois. Doucement. L'eau est fraîche. Une feuille tourne près du pied. Le jardin, il a vu. La soupe, maintenant ! On rentre. Je cours ! Amir veut foncer vers la porte. La gourde a roulé près de la feuille. La casquette est sur une chaise basse. Le sourire d'Amir se serre. Ça serre, dans son ventre. Je n'aime pas ça. Amir refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Amir observe la gourde, écoute le jardin. Dans l'eau, un éclat blanc tremble. Comme l'&lt;emphasis level="moderate"&gt;éclat de casserole&lt;/emphasis&gt;, maman ! Tu le vois, celui-là ? Oui, maman. Il pointe le lapin. Il contourne la feuille, lentement. Il reprend la gourde près de la feuille. Il reprend la casquette, sur la chaise. Et le lapin. Le doudou est dans son bras. Tu tiens le lapin ? Oui, il a voyagé.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Benoît marche près de maman. Le doudou est dans son bras. [pause]</t>
+          <t>Plus tard, ils jouent au jardin. L'odeur de soupe passe sous la porte. Amir a une gourde. Il a une casquette. Le lapin est dans l'herbe courte. Je bois. Doucement. L'eau est fraîche. Une feuille tourne près du pied. Le jardin, il a vu. La soupe, maintenant ! On rentre. Je cours ! Amir veut foncer vers la porte. La gourde a roulé près de la feuille. La casquette est sur une chaise basse. Le sourire d'Amir se serre. Ça serre, dans son ventre. Je n'aime pas ça. Amir refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Amir observe la gourde, écoute le jardin. Dans l'eau, un éclat blanc tremble. Comme l'&lt;emphasis&gt;éclat de casserole&lt;/emphasis&gt;, maman ! Tu le vois, celui-là ? Oui, maman. Il pointe le lapin. Il contourne la feuille, lentement. Il reprend la gourde près de la feuille. Il reprend la casquette, sur la chaise. Et le lapin. Le doudou est dans son bras. Tu tiens le lapin ? Oui, il a voyagé. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1866,7 +1855,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1874,10 +1863,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1898,28 +1887,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de casserole</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1928,10 +1921,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1942,27 +1935,53 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_vers_la_soupe; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Amir marche près de maman.
+          <t>narrateur|Plus tard, ils jouent au jardin.
+narrateur|L'odeur de soupe passe sous la porte.
+narrateur|Amir a une gourde.
+narrateur|Il a une casquette.
+narrateur|Le lapin est dans l'herbe courte.
+enfant-m|Je bois.
+maman|Doucement.
+narrateur|L'eau est fraîche.
+narrateur|Une feuille tourne près du pied.
+enfant-m|Le jardin, il a vu.
+enfant-m|La soupe, maintenant !
+maman|On rentre.
+enfant-m|Je cours !
+narrateur|Amir veut foncer vers la porte.
+narrateur|La gourde a roulé près de la feuille.
+narrateur|La casquette est sur une chaise basse.
+narrateur|Le sourire d'Amir se serre.
+narrateur|Ça serre, dans son ventre.
+enfant-m|Je n'aime pas ça.
+narrateur|Amir refuse de foncer.
+enfant-m|Attends, je regarde.
+narrateur|Personne ne donne la réponse.
+narrateur|Amir observe la gourde, écoute le jardin.
+narrateur|Dans l'eau, un éclat blanc tremble.
+enfant-m|Comme l'éclat de casserole, maman !
+maman|Tu le vois, celui-là ?
+enfant-m|Oui, maman.
+enfant-m|Il pointe le lapin.
+narrateur|Il contourne la feuille, lentement.
+narrateur|Il reprend la gourde près de la feuille.
+narrateur|Il reprend la casquette, sur la chaise.
+enfant-m|Et le lapin.
 narrateur|Le doudou est dans son bras.
-narrateur|Ils ouvrent la porte.
-narrateur|La soupe sent encore plus fort.
-maman|Tu poses la gourde près de l'évier ?
-narrateur|Amir pose la gourde.
-narrateur|Il pose la casquette.
-maman|Merci.
-maman|Ce soir, on mange la soupe.
-enfant-m|Carotte et poireau.
-maman|Oui.
-narrateur|Amir pose le lapin sur une chaise.
-enfant-m|Il a vu le parc.
-enfant-m|Il a vu le jardin.
-maman|Et maintenant, la soupe.
-narrateur|Un peu de vapeur monte.
-enfant-m|Il goûte l'odeur.
-maman|Tout doux.</t>
+maman|Tu tiens le lapin ?
+enfant-m|Oui, il a voyagé.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>herbe,gourde</t>
         </is>
       </c>
     </row>
@@ -1989,17 +2008,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le lapin a voyagé. Et toi, tu as repris tes affaires. La casserole est encore tiède.</t>
+          <t>Ils ouvrent la porte de la cuisine. La soupe sent plus fort. Tu poses la gourde près de l'évier ? Amir pose la gourde. Il pose la casquette. La soupe. Oui, carotte et poireau. Amir pose le lapin sur une chaise. Il a vu le parc. Il a vu le jardin. Et maintenant, la soupe. Un peu de vapeur monte. Mon éclat de casserole, maman. Sur le bord, l'éclat de casserole brille. Le fil de vapeur passe devant. Ils se regardent. Tu les sens, la soupe et le lapin ? Oui, maman. La soupe sent le chaud. L'éclat de casserole reste sur le bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le lapin a voyagé. Et toi, tu as repris tes affaires. La casserole est encore tiède.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils ouvrent la porte de la cuisine. La soupe sent plus fort. Tu poses la gourde près de l'évier ? Amir pose la gourde. Il pose la casquette. La soupe. Oui, carotte et poireau. Amir pose le lapin sur une chaise. Il a vu le parc. Il a vu le jardin. Et maintenant, la soupe. Un peu de vapeur monte. Mon &lt;emphasis level="moderate"&gt;éclat de casserole&lt;/emphasis&gt;, maman. Sur le bord, l'éclat de casserole brille. Le fil de vapeur passe devant. Ils se regardent. Tu les sens, la soupe et le lapin ? Oui, maman. La soupe sent le chaud. L'éclat de casserole reste sur le bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils ouvrent la porte de la cuisine. La soupe sent plus fort. Tu poses la gourde près de l'évier ? Amir pose la gourde. Il pose la casquette. La soupe. Oui, carotte et poireau. Amir pose le lapin sur une chaise. Il a vu le parc. Il a vu le jardin. Et maintenant, la soupe. Un peu de vapeur monte. Mon &lt;emphasis&gt;éclat de casserole&lt;/emphasis&gt;, maman. Sur le bord, l'éclat de casserole brille. Le fil de vapeur passe devant. Ils se regardent. Tu les sens, la soupe et le lapin ? Oui, maman. La soupe sent le chaud. L'éclat de casserole reste sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2046,18 +2065,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2066,12 +2085,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2080,17 +2099,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de casserole</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2099,11 +2122,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2112,26 +2135,52 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_casserole_est_sur_le_bord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Le lapin a voyagé.
-maman|Et toi, tu as repris tes affaires.
-narrateur|La casserole est encore tiède.</t>
+          <t>narrateur|Ils ouvrent la porte de la cuisine.
+narrateur|La soupe sent plus fort.
+maman|Tu poses la gourde près de l'évier ?
+narrateur|Amir pose la gourde.
+narrateur|Il pose la casquette.
+enfant-m|La soupe.
+maman|Oui, carotte et poireau.
+narrateur|Amir pose le lapin sur une chaise.
+enfant-m|Il a vu le parc.
+enfant-m|Il a vu le jardin.
+maman|Et maintenant, la soupe.
+narrateur|Un peu de vapeur monte.
+enfant-m|Mon éclat de casserole, maman.
+narrateur|Sur le bord, l'éclat de casserole brille.
+narrateur|Le fil de vapeur passe devant.
+enfant-m|Ils se regardent.
+maman|Tu les sens, la soupe et le lapin ?
+enfant-m|Oui, maman.
+enfant-m|La soupe sent le chaud.
+narrateur|L'éclat de casserole reste sur le bord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>soupe,casserole</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2244,6 +2293,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>